<commit_message>
bank cash report ui updated
</commit_message>
<xml_diff>
--- a/nexus_river_view_master.xlsx
+++ b/nexus_river_view_master.xlsx
@@ -2129,11 +2129,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H92"/>
+  <dimension ref="A1:H93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="646" customWidth="1" min="2" max="2"/>
+    <col width="278" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
@@ -5202,16 +5202,13 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Voucher DV38: 22.06.2026 – Visited Jahid Sir's office for cheque signing.And Modhu Hazi office Transportation expense: Tk. 120.
-23.06.2026 – Visited Modhu Hazi River View Project to discuss the location for the labour shed. Transportation expense: Tk. 100.
-24.06.2026 – Visited Modhu Hazi River View Project and Ati Bazar to discuss the estimated expenses for the labour shed and submersible pump. Transportation expense: Tk. 130.
-25.06.2026 – Visited Modu City Electric Office to deposit transformer-related funds and later visited Modhu Hazi River View Project to discuss labour shed work with the mason. Transportation expense: Tk. 120.
+          <t xml:space="preserve">Voucher DV40: Entertainment cost for meeting 25 June 2026                        
 </t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Conveyance</t>
+          <t>Entertainment</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -5223,10 +5220,10 @@
         <v>0</v>
       </c>
       <c r="F90" t="n">
-        <v>470</v>
+        <v>5030</v>
       </c>
       <c r="G90" t="n">
-        <v>82773</v>
+        <v>78213</v>
       </c>
       <c r="H90" t="inlineStr"/>
     </row>
@@ -5238,13 +5235,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Voucher DV40: Entertainment cost for meeting 25 June 2026                        
-</t>
+          <t>Voucher DV39: TS Transformer Purchase Cost for Electricity Line</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Entertainment</t>
+          <t>Electric</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -5256,44 +5252,76 @@
         <v>0</v>
       </c>
       <c r="F91" t="n">
-        <v>5030</v>
+        <v>84500</v>
       </c>
       <c r="G91" t="n">
-        <v>77743</v>
+        <v>-6287</v>
       </c>
       <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Voucher DV39: TS Transformer Purchase Cost for Electricity Line</t>
+          <t>Contra CN16: Entertainmnet , Conveyance , Stationary , pretty cash (Transfer from Bank)</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Electric</t>
+          <t>Contra</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92" t="n">
+        <v>3713</v>
+      </c>
+      <c r="H92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Voucher DV38: 6 Days' Conveyance Expense of Shariful</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Conveyance</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="E92" t="n">
-        <v>0</v>
-      </c>
-      <c r="F92" t="n">
-        <v>84500</v>
-      </c>
-      <c r="G92" t="n">
-        <v>-6757</v>
-      </c>
-      <c r="H92" t="inlineStr"/>
+      <c r="E93" t="n">
+        <v>0</v>
+      </c>
+      <c r="F93" t="n">
+        <v>670</v>
+      </c>
+      <c r="G93" t="n">
+        <v>3043</v>
+      </c>
+      <c r="H93" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7046,7 +7074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8258,7 +8286,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -8271,17 +8299,17 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Trn. Br: 000 000245******0000 00600009 000841231133</t>
+          <t>Contra CN16: Transfer to Cash</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="F42" t="n">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>1820655.49</v>
+        <v>1129195.49</v>
       </c>
     </row>
     <row r="43">
@@ -8300,7 +8328,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Trn. Br: 084 AGBKBDDH, JATIYA PRESS CLUB, MD ATAUR RAHMAN CHOWDHURY - PAYMENT - SCCT</t>
+          <t>Trn. Br: 000 000245******0000 00600009 000841231133</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -8310,7 +8338,7 @@
         <v>100000</v>
       </c>
       <c r="G43" t="n">
-        <v>1920655.49</v>
+        <v>1820655.49</v>
       </c>
     </row>
     <row r="44">
@@ -8329,7 +8357,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Trn. Br: 084 IBBLBDDH, UTTARA, Shahidul Islam -</t>
+          <t>Trn. Br: 084 AGBKBDDH, JATIYA PRESS CLUB, MD ATAUR RAHMAN CHOWDHURY - PAYMENT - SCCT</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -8339,13 +8367,13 @@
         <v>100000</v>
       </c>
       <c r="G44" t="n">
-        <v>2020655.49</v>
+        <v>1920655.49</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -8358,7 +8386,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Trn. Br: 000 000245******0000 00600009 000842082313</t>
+          <t>Trn. Br: 084 IBBLBDDH, UTTARA, Shahidul Islam -</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -8368,13 +8396,13 @@
         <v>100000</v>
       </c>
       <c r="G45" t="n">
-        <v>2120655.49</v>
+        <v>2020655.49</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -8387,17 +8415,17 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Trn. Br: 084</t>
+          <t>Trn. Br: 000 000245******0000 00600009 000842082313</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="G46" t="n">
-        <v>50700</v>
+        <v>2120655.49</v>
       </c>
     </row>
     <row r="47">
@@ -8420,19 +8448,19 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>45</v>
+        <v>300</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>50655</v>
+        <v>50700</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -8445,23 +8473,23 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Trn. Br: 084 IBBLBDDH, FENI, MOHAMMED JAHIR ULLAH -</t>
+          <t>Trn. Br: 084</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F48" t="n">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="G48" t="n">
-        <v>2320655.49</v>
+        <v>50655</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -8474,23 +8502,23 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">	Banking Fund Transfer - Credit</t>
+          <t>Trn. Br: 084 IBBLBDDH, FENI, MOHAMMED JAHIR ULLAH -</t>
         </is>
       </c>
       <c r="E49" t="n">
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>100000</v>
+        <v>200000</v>
       </c>
       <c r="G49" t="n">
-        <v>4214145.49</v>
+        <v>2320655.49</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -8503,7 +8531,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Trn. Br: 084 ISLAMI BANK BANGLDESH LTD., AGENT BANKING Related Account: 0843201000809046</t>
+          <t xml:space="preserve">	Banking Fund Transfer - Credit</t>
         </is>
       </c>
       <c r="E50" t="n">
@@ -8513,7 +8541,7 @@
         <v>100000</v>
       </c>
       <c r="G50" t="n">
-        <v>2420655.49</v>
+        <v>4214145.49</v>
       </c>
     </row>
     <row r="51">
@@ -8536,13 +8564,13 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="G51" t="n">
-        <v>2420645.49</v>
+        <v>2420655.49</v>
       </c>
     </row>
     <row r="52">
@@ -8561,23 +8589,23 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Trn. Br: 777 IB(Unet) pay</t>
+          <t>Trn. Br: 084 ISLAMI BANK BANGLDESH LTD., AGENT BANKING Related Account: 0843201000809046</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F52" t="n">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>2620645.49</v>
+        <v>2420645.49</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -8590,23 +8618,23 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Banking Fund Transfer - Credit</t>
+          <t>Trn. Br: 777 IB(Unet) pay</t>
         </is>
       </c>
       <c r="E53" t="n">
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>500000</v>
+        <v>200000</v>
       </c>
       <c r="G53" t="n">
-        <v>4714145.49</v>
+        <v>2620645.49</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -8619,17 +8647,17 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Trn. Br: 084 SUMIYA BINTE SHAHID 2706101119862 Alimuzzman-ID: B17526027A326697 _Pubali Bank PLC, TRUNCATION POINT</t>
+          <t>Banking Fund Transfer - Credit</t>
         </is>
       </c>
       <c r="E54" t="n">
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>90000</v>
+        <v>500000</v>
       </c>
       <c r="G54" t="n">
-        <v>2710645.49</v>
+        <v>4714145.49</v>
       </c>
     </row>
     <row r="55">
@@ -8648,17 +8676,17 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Trn. Br: 084 ALIMUZZAMAN 1161030187123 Alimuzzman-ID: B09026027A030590 _Dutch-Bangla Bank PLC,LOCAL OFFICE</t>
+          <t>Trn. Br: 084 SUMIYA BINTE SHAHID 2706101119862 Alimuzzman-ID: B17526027A326697 _Pubali Bank PLC, TRUNCATION POINT</t>
         </is>
       </c>
       <c r="E55" t="n">
         <v>0</v>
       </c>
       <c r="F55" t="n">
-        <v>110000</v>
+        <v>90000</v>
       </c>
       <c r="G55" t="n">
-        <v>2820645.49</v>
+        <v>2710645.49</v>
       </c>
     </row>
     <row r="56">
@@ -8677,17 +8705,17 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Trn. Br: 084 SUSMITA DAS 0100007463043 1st Installment N-ID: B13526027O074980 _JANATA BANK LTD..HEAD OFFICE</t>
+          <t>Trn. Br: 084 ALIMUZZAMAN 1161030187123 Alimuzzman-ID: B09026027A030590 _Dutch-Bangla Bank PLC,LOCAL OFFICE</t>
         </is>
       </c>
       <c r="E56" t="n">
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>100000</v>
+        <v>110000</v>
       </c>
       <c r="G56" t="n">
-        <v>2920645.49</v>
+        <v>2820645.49</v>
       </c>
     </row>
     <row r="57">
@@ -8706,7 +8734,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Trn. Br: 000 000245******0000 90001000 000845920253</t>
+          <t>Trn. Br: 084 SUSMITA DAS 0100007463043 1st Installment N-ID: B13526027O074980 _JANATA BANK LTD..HEAD OFFICE</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -8716,13 +8744,13 @@
         <v>100000</v>
       </c>
       <c r="G57" t="n">
-        <v>3020645.49</v>
+        <v>2920645.49</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -8735,17 +8763,17 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Trn. Br: 786 EB (Unet)businesses</t>
+          <t>Trn. Br: 000 000245******0000 90001000 000845920253</t>
         </is>
       </c>
       <c r="E58" t="n">
         <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>300000</v>
+        <v>100000</v>
       </c>
       <c r="G58" t="n">
-        <v>3320645.49</v>
+        <v>3020645.49</v>
       </c>
     </row>
     <row r="59">
@@ -8764,23 +8792,23 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Trn. Br: 786 EB (Unet)Business</t>
+          <t>Trn. Br: 786 EB (Unet)businesses</t>
         </is>
       </c>
       <c r="E59" t="n">
         <v>0</v>
       </c>
       <c r="F59" t="n">
-        <v>100000</v>
+        <v>300000</v>
       </c>
       <c r="G59" t="n">
-        <v>3420645.49</v>
+        <v>3320645.49</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -8793,17 +8821,17 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Trn. Br: 084 Related Account: 0843201000809046</t>
+          <t>Trn. Br: 786 EB (Unet)Business</t>
         </is>
       </c>
       <c r="E60" t="n">
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>0.58</v>
+        <v>100000</v>
       </c>
       <c r="G60" t="n">
-        <v>50655.58</v>
+        <v>3420645.49</v>
       </c>
     </row>
     <row r="61">
@@ -8826,12 +8854,41 @@
         </is>
       </c>
       <c r="E61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G61" t="n">
+        <v>50655.58</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>31-12-2025</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>United Commercial Bank PLC</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Trn. Br: 084 Related Account: 0843201000809046</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
         <v>0.09</v>
       </c>
-      <c r="F61" t="n">
-        <v>0</v>
-      </c>
-      <c r="G61" t="n">
+      <c r="F62" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" t="n">
         <v>50655.49</v>
       </c>
     </row>

</xml_diff>